<commit_message>
feat(mobile): in-app language selector + patrol report fixes
- Add Settings -> Language picker (English, Hindi, Telugu, Bengali) with
  runtime locale switching via ContextWrapper; localize bottom-nav labels
  through nav_* string resources.
- Fix End Patrol button staying after ending: navigation no longer blocked
  by sync errors and ended state is reflected immediately.
- Anchor patrol end time to the real stop time (trusted timer) instead of the
  last GPS sample, so duration reflects true start->end rather than collapsing
  to ~2 minutes.
- Persist patrol team details on a scope that survives navigation so they
  appear in the report instead of a constant "Loading..." subtitle.

Co-Authored-By: opencode <noreply@opencode.ai>
</commit_message>
<xml_diff>
--- a/docs/work_plan.xlsx
+++ b/docs/work_plan.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -822,18 +822,18 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>UI + now persists local session and creates backend patrol at start.</t>
+          <t>UI + reliably persists local session (team details) so they appear in PatrolReportScreen; creates backend patrol at start.</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>End time + stats persisted on stop (ActivitySummary) and POSTed to /api/patrols/:id/complete; shown in PatrolReportScreen timing section.</t>
+          <t>End time + stats persisted on stop and POSTed to /api/patrols/:id/complete. End time now anchored to the real patrol stop time (trusted timer) instead of the last GPS sample, so duration reflects true start-&gt;end (fixes collapsed ~2-min durations). End Patrol button now hides immediately on confirm and navigation is not blocked by sync errors.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>PatrolReportScreen falls back to GET /api/patrols/:id (+stats) when no local session; renders summary/timing/team. Route map still local-only (no GET points endpoint).</t>
+          <t>Falls back to GET /api/patrols/:id when no local session; renders summary/timing/team. Team details + duration now correct (local session persistence + real end time fixed this session). Route map still local-only (no GET points endpoint).</t>
         </is>
       </c>
     </row>
@@ -2270,6 +2270,72 @@
       <c r="G55" s="4" t="inlineStr">
         <is>
           <t>Real-device forest test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>K01</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Localization &amp; i18n</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>In-app language selector (Settings -&gt; Language)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>100</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Settings -&gt; Language offers English, Hindi, Telugu, Bengali; runtime locale switch via ContextWrapper; bottom-nav labels localized through nav_* string resources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>K02</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Localization &amp; i18n</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Translated string resources (hi/te/bn)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>70</v>
+      </c>
+      <c r="F57" t="n">
+        <v>3</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>nav_*, settings and core strings translated; full catalog coverage still pending.</t>
         </is>
       </c>
     </row>

</xml_diff>